<commit_message>
Refactor ManageModels: Baseline logic, Reset year range, and UI improvements
- Replace all references of "BAU" with "Baseline" in carbon credits and Excel outputs.

- Update Excel files to show "vs Baseline" instead of "vs BAU".

- Removed logic for creating BAU model, instead defining year range for scenario

- Implement Reset Year Range button to delete the Baseline model, with confirmation dialog.

- Display current scenario year range next to the reset button.

- Adjust logic to show "No techno-economic models available" only when no models besides Baseline exist.

- Ensure model creation form handles Baseline separately and protects reserved name.
</commit_message>
<xml_diff>
--- a/backend/Rwanda/carbon-credits-{template}.xlsx
+++ b/backend/Rwanda/carbon-credits-{template}.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8954da175e61d5af/Escritorio/IIT/CC-WBT/backend/{templates}/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{4007055A-7FB8-4884-B6C5-AD44DAA53F1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{44AD9C85-B674-423A-9687-93095E623D13}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="13_ncr:1_{4007055A-7FB8-4884-B6C5-AD44DAA53F1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FDF2BEA4-3B9E-4B8D-ACAC-A396EE65C4A5}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,9 +41,6 @@
     <t>Units</t>
   </si>
   <si>
-    <t>CO2 emited - BAU scenario</t>
-  </si>
-  <si>
     <t>CO2Eq MT/y</t>
   </si>
   <si>
@@ -53,9 +50,6 @@
     <t>CO2 emited - {model} scenario</t>
   </si>
   <si>
-    <t>△▲{model} vs. BAU</t>
-  </si>
-  <si>
     <t>CO2 equivalent avoided in the {model}</t>
   </si>
   <si>
@@ -63,6 +57,12 @@
   </si>
   <si>
     <t>Inputs</t>
+  </si>
+  <si>
+    <t>△▲{model} vs. Baseline</t>
+  </si>
+  <si>
+    <t>CO2 emited - Baseline scenario</t>
   </si>
 </sst>
 </file>
@@ -218,6 +218,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -494,7 +498,7 @@
   <sheetData>
     <row r="1" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B1" s="6" t="s">
         <v>0</v>
@@ -626,10 +630,10 @@
     </row>
     <row r="2" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>1</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>2</v>
       </c>
       <c r="C2" s="11">
         <v>0</v>
@@ -758,10 +762,10 @@
     </row>
     <row r="3" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3" s="11">
         <v>0</v>
@@ -890,10 +894,10 @@
     </row>
     <row r="4" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C4" s="11">
         <v>0</v>
@@ -1022,10 +1026,10 @@
     </row>
     <row r="5" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C5" s="11">
         <v>0</v>
@@ -1154,10 +1158,10 @@
     </row>
     <row r="6" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C6" s="11">
         <v>0</v>

</xml_diff>

<commit_message>
Refactor Carbon Credits section and improve accessibility
- Refactored the Carbon Credits section structure and logic

- Made the Carbon Credits button globally accessible across the platform
  (functionality enabled without having a model selected)

- Moved Carbon Credits to the Outputs section, as it is an additional feature  that does not affect core output calculations (e.g. FFSS)

- Reworked the conceptual foundations to be scenario-agnostic and always accessible

- Enabled annual CO2 emissions inputs for all models, including the baseline

- Used these inputs to compute projections such as CO2 avoided and potential income
</commit_message>
<xml_diff>
--- a/backend/Rwanda/carbon-credits-{template}.xlsx
+++ b/backend/Rwanda/carbon-credits-{template}.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8954da175e61d5af/Escritorio/IIT/CC-WBT/backend/{templates}/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8954da175e61d5af/Escritorio/IIT/CC-WBT/backend/Rwanda/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="13_ncr:1_{4007055A-7FB8-4884-B6C5-AD44DAA53F1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FDF2BEA4-3B9E-4B8D-ACAC-A396EE65C4A5}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="13_ncr:1_{4007055A-7FB8-4884-B6C5-AD44DAA53F1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9119E20A-1FCD-48CA-8469-ED096C8CCBF0}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="10">
   <si>
     <t>Units</t>
   </si>
@@ -56,13 +56,16 @@
     <t>Potential income from Carbon Credits in the {model} Plan - right</t>
   </si>
   <si>
-    <t>Inputs</t>
-  </si>
-  <si>
     <t>△▲{model} vs. Baseline</t>
   </si>
   <si>
     <t>CO2 emited - Baseline scenario</t>
+  </si>
+  <si>
+    <t>CO2 Inputs</t>
+  </si>
+  <si>
+    <t>Carbon Credits</t>
   </si>
 </sst>
 </file>
@@ -218,10 +221,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -488,7 +487,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99682AE1-5334-4A99-9652-64DF807A4E7D}">
   <sheetPr codeName="Hoja2"/>
-  <dimension ref="A1:AR8"/>
+  <dimension ref="A1:AR9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="59.54296875" customWidth="1"/>
@@ -498,7 +497,7 @@
   <sheetData>
     <row r="1" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B1" s="6" t="s">
         <v>0</v>
@@ -630,7 +629,7 @@
     </row>
     <row r="2" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>1</v>
@@ -893,140 +892,140 @@
       <c r="AR3" s="8"/>
     </row>
     <row r="4" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" s="11">
-        <v>0</v>
-      </c>
-      <c r="D4" s="11">
-        <v>0</v>
-      </c>
-      <c r="E4" s="11">
-        <v>0</v>
-      </c>
-      <c r="F4" s="11">
-        <v>0</v>
-      </c>
-      <c r="G4" s="11">
-        <v>0</v>
-      </c>
-      <c r="H4" s="11">
-        <v>0</v>
-      </c>
-      <c r="I4" s="11">
-        <v>0</v>
-      </c>
-      <c r="J4" s="11">
-        <v>0</v>
-      </c>
-      <c r="K4" s="11">
-        <v>0</v>
-      </c>
-      <c r="L4" s="11">
-        <v>0</v>
-      </c>
-      <c r="M4" s="11">
-        <v>0</v>
-      </c>
-      <c r="N4" s="11">
-        <v>0</v>
-      </c>
-      <c r="O4" s="11">
-        <v>0</v>
-      </c>
-      <c r="P4" s="11">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="11">
-        <v>0</v>
-      </c>
-      <c r="R4" s="11">
-        <v>0</v>
-      </c>
-      <c r="S4" s="11">
-        <v>0</v>
-      </c>
-      <c r="T4" s="11">
-        <v>0</v>
-      </c>
-      <c r="U4" s="11">
-        <v>0</v>
-      </c>
-      <c r="V4" s="11">
-        <v>0</v>
-      </c>
-      <c r="W4" s="11">
-        <v>0</v>
-      </c>
-      <c r="X4" s="11">
-        <v>0</v>
-      </c>
-      <c r="Y4" s="11">
-        <v>0</v>
-      </c>
-      <c r="Z4" s="11">
-        <v>0</v>
-      </c>
-      <c r="AA4" s="11">
-        <v>0</v>
-      </c>
-      <c r="AB4" s="11">
-        <v>0</v>
-      </c>
-      <c r="AC4" s="11">
-        <v>0</v>
-      </c>
-      <c r="AD4" s="11">
-        <v>0</v>
-      </c>
-      <c r="AE4" s="11">
-        <v>0</v>
-      </c>
-      <c r="AF4" s="11">
-        <v>0</v>
-      </c>
-      <c r="AG4" s="11">
-        <v>0</v>
-      </c>
-      <c r="AH4" s="11">
-        <v>0</v>
-      </c>
-      <c r="AI4" s="11">
-        <v>0</v>
-      </c>
-      <c r="AJ4" s="11">
-        <v>0</v>
-      </c>
-      <c r="AK4" s="11">
-        <v>0</v>
-      </c>
-      <c r="AL4" s="11">
-        <v>0</v>
-      </c>
-      <c r="AM4" s="11">
-        <v>0</v>
-      </c>
-      <c r="AN4" s="11">
-        <v>0</v>
-      </c>
-      <c r="AO4" s="11">
-        <v>0</v>
-      </c>
-      <c r="AP4" s="11">
-        <v>0</v>
-      </c>
-      <c r="AQ4" s="11">
-        <v>0</v>
+      <c r="A4" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="7">
+        <v>2020</v>
+      </c>
+      <c r="D4" s="7">
+        <v>2021</v>
+      </c>
+      <c r="E4" s="7">
+        <v>2022</v>
+      </c>
+      <c r="F4" s="7">
+        <v>2023</v>
+      </c>
+      <c r="G4" s="7">
+        <v>2024</v>
+      </c>
+      <c r="H4" s="7">
+        <v>2025</v>
+      </c>
+      <c r="I4" s="7">
+        <v>2026</v>
+      </c>
+      <c r="J4" s="7">
+        <v>2027</v>
+      </c>
+      <c r="K4" s="7">
+        <v>2028</v>
+      </c>
+      <c r="L4" s="7">
+        <v>2029</v>
+      </c>
+      <c r="M4" s="7">
+        <v>2030</v>
+      </c>
+      <c r="N4" s="7">
+        <v>2031</v>
+      </c>
+      <c r="O4" s="7">
+        <v>2032</v>
+      </c>
+      <c r="P4" s="7">
+        <v>2033</v>
+      </c>
+      <c r="Q4" s="7">
+        <v>2034</v>
+      </c>
+      <c r="R4" s="7">
+        <v>2035</v>
+      </c>
+      <c r="S4" s="7">
+        <v>2036</v>
+      </c>
+      <c r="T4" s="7">
+        <v>2037</v>
+      </c>
+      <c r="U4" s="7">
+        <v>2038</v>
+      </c>
+      <c r="V4" s="7">
+        <v>2039</v>
+      </c>
+      <c r="W4" s="7">
+        <v>2040</v>
+      </c>
+      <c r="X4" s="7">
+        <v>2041</v>
+      </c>
+      <c r="Y4" s="7">
+        <v>2042</v>
+      </c>
+      <c r="Z4" s="7">
+        <v>2043</v>
+      </c>
+      <c r="AA4" s="7">
+        <v>2044</v>
+      </c>
+      <c r="AB4" s="7">
+        <v>2045</v>
+      </c>
+      <c r="AC4" s="7">
+        <v>2046</v>
+      </c>
+      <c r="AD4" s="7">
+        <v>2047</v>
+      </c>
+      <c r="AE4" s="7">
+        <v>2048</v>
+      </c>
+      <c r="AF4" s="7">
+        <v>2049</v>
+      </c>
+      <c r="AG4" s="7">
+        <v>2050</v>
+      </c>
+      <c r="AH4" s="7">
+        <v>2051</v>
+      </c>
+      <c r="AI4" s="7">
+        <v>2052</v>
+      </c>
+      <c r="AJ4" s="7">
+        <v>2053</v>
+      </c>
+      <c r="AK4" s="7">
+        <v>2054</v>
+      </c>
+      <c r="AL4" s="7">
+        <v>2055</v>
+      </c>
+      <c r="AM4" s="7">
+        <v>2056</v>
+      </c>
+      <c r="AN4" s="7">
+        <v>2057</v>
+      </c>
+      <c r="AO4" s="7">
+        <v>2058</v>
+      </c>
+      <c r="AP4" s="7">
+        <v>2059</v>
+      </c>
+      <c r="AQ4" s="7">
+        <v>2060</v>
       </c>
       <c r="AR4" s="8"/>
     </row>
     <row r="5" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>1</v>
@@ -1158,10 +1157,10 @@
     </row>
     <row r="6" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C6" s="11">
         <v>0</v>
@@ -1289,66 +1288,198 @@
       <c r="AR6" s="8"/>
     </row>
     <row r="7" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="9"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="10"/>
-      <c r="G7" s="10"/>
-      <c r="H7" s="10"/>
-      <c r="I7" s="10"/>
-      <c r="J7" s="10"/>
-      <c r="K7" s="10"/>
-      <c r="L7" s="10"/>
-      <c r="M7" s="10"/>
-      <c r="N7" s="10"/>
-      <c r="O7" s="10"/>
-      <c r="P7" s="10"/>
-      <c r="Q7" s="10"/>
-      <c r="R7" s="10"/>
-      <c r="S7" s="10"/>
-      <c r="T7" s="10"/>
-      <c r="U7" s="10"/>
-      <c r="V7" s="10"/>
-      <c r="W7" s="10"/>
-      <c r="X7" s="10"/>
-      <c r="Y7" s="10"/>
-      <c r="Z7" s="10"/>
-      <c r="AA7" s="10"/>
-      <c r="AB7" s="10"/>
-      <c r="AC7" s="10"/>
-      <c r="AD7" s="10"/>
-      <c r="AE7" s="10"/>
-      <c r="AF7" s="10"/>
-      <c r="AG7" s="10"/>
-      <c r="AH7" s="8"/>
-      <c r="AI7" s="8"/>
-      <c r="AJ7" s="8"/>
-      <c r="AK7" s="8"/>
-      <c r="AL7" s="8"/>
-      <c r="AM7" s="8"/>
-      <c r="AN7" s="8"/>
-      <c r="AO7" s="8"/>
-      <c r="AP7" s="8"/>
-      <c r="AQ7" s="8"/>
+      <c r="A7" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C7" s="11">
+        <v>0</v>
+      </c>
+      <c r="D7" s="11">
+        <v>0</v>
+      </c>
+      <c r="E7" s="11">
+        <v>0</v>
+      </c>
+      <c r="F7" s="11">
+        <v>0</v>
+      </c>
+      <c r="G7" s="11">
+        <v>0</v>
+      </c>
+      <c r="H7" s="11">
+        <v>0</v>
+      </c>
+      <c r="I7" s="11">
+        <v>0</v>
+      </c>
+      <c r="J7" s="11">
+        <v>0</v>
+      </c>
+      <c r="K7" s="11">
+        <v>0</v>
+      </c>
+      <c r="L7" s="11">
+        <v>0</v>
+      </c>
+      <c r="M7" s="11">
+        <v>0</v>
+      </c>
+      <c r="N7" s="11">
+        <v>0</v>
+      </c>
+      <c r="O7" s="11">
+        <v>0</v>
+      </c>
+      <c r="P7" s="11">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="11">
+        <v>0</v>
+      </c>
+      <c r="R7" s="11">
+        <v>0</v>
+      </c>
+      <c r="S7" s="11">
+        <v>0</v>
+      </c>
+      <c r="T7" s="11">
+        <v>0</v>
+      </c>
+      <c r="U7" s="11">
+        <v>0</v>
+      </c>
+      <c r="V7" s="11">
+        <v>0</v>
+      </c>
+      <c r="W7" s="11">
+        <v>0</v>
+      </c>
+      <c r="X7" s="11">
+        <v>0</v>
+      </c>
+      <c r="Y7" s="11">
+        <v>0</v>
+      </c>
+      <c r="Z7" s="11">
+        <v>0</v>
+      </c>
+      <c r="AA7" s="11">
+        <v>0</v>
+      </c>
+      <c r="AB7" s="11">
+        <v>0</v>
+      </c>
+      <c r="AC7" s="11">
+        <v>0</v>
+      </c>
+      <c r="AD7" s="11">
+        <v>0</v>
+      </c>
+      <c r="AE7" s="11">
+        <v>0</v>
+      </c>
+      <c r="AF7" s="11">
+        <v>0</v>
+      </c>
+      <c r="AG7" s="11">
+        <v>0</v>
+      </c>
+      <c r="AH7" s="11">
+        <v>0</v>
+      </c>
+      <c r="AI7" s="11">
+        <v>0</v>
+      </c>
+      <c r="AJ7" s="11">
+        <v>0</v>
+      </c>
+      <c r="AK7" s="11">
+        <v>0</v>
+      </c>
+      <c r="AL7" s="11">
+        <v>0</v>
+      </c>
+      <c r="AM7" s="11">
+        <v>0</v>
+      </c>
+      <c r="AN7" s="11">
+        <v>0</v>
+      </c>
+      <c r="AO7" s="11">
+        <v>0</v>
+      </c>
+      <c r="AP7" s="11">
+        <v>0</v>
+      </c>
+      <c r="AQ7" s="11">
+        <v>0</v>
+      </c>
       <c r="AR7" s="8"/>
     </row>
     <row r="8" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="2"/>
+      <c r="A8" s="9"/>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
-      <c r="N8" s="2"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="10"/>
+      <c r="J8" s="10"/>
+      <c r="K8" s="10"/>
+      <c r="L8" s="10"/>
+      <c r="M8" s="10"/>
+      <c r="N8" s="10"/>
+      <c r="O8" s="10"/>
+      <c r="P8" s="10"/>
+      <c r="Q8" s="10"/>
+      <c r="R8" s="10"/>
+      <c r="S8" s="10"/>
+      <c r="T8" s="10"/>
+      <c r="U8" s="10"/>
+      <c r="V8" s="10"/>
+      <c r="W8" s="10"/>
+      <c r="X8" s="10"/>
+      <c r="Y8" s="10"/>
+      <c r="Z8" s="10"/>
+      <c r="AA8" s="10"/>
+      <c r="AB8" s="10"/>
+      <c r="AC8" s="10"/>
+      <c r="AD8" s="10"/>
+      <c r="AE8" s="10"/>
+      <c r="AF8" s="10"/>
+      <c r="AG8" s="10"/>
+      <c r="AH8" s="8"/>
+      <c r="AI8" s="8"/>
+      <c r="AJ8" s="8"/>
+      <c r="AK8" s="8"/>
+      <c r="AL8" s="8"/>
+      <c r="AM8" s="8"/>
+      <c r="AN8" s="8"/>
+      <c r="AO8" s="8"/>
+      <c r="AP8" s="8"/>
+      <c r="AQ8" s="8"/>
+      <c r="AR8" s="8"/>
+    </row>
+    <row r="9" spans="1:44" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A9" s="2"/>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2"/>
+      <c r="J9" s="2"/>
+      <c r="K9" s="2"/>
+      <c r="L9" s="2"/>
+      <c r="M9" s="2"/>
+      <c r="N9" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>